<commit_message>
Finalized PCB Schematic and PCB
</commit_message>
<xml_diff>
--- a/Components_list.xlsx
+++ b/Components_list.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="97" documentId="11_F25DC773A252ABDACC1048B781584E2E5BDE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6FB6178F-0E14-4B57-B366-0D5AB7865750}"/>
   <bookViews>
-    <workbookView xWindow="-60" yWindow="-60" windowWidth="21720" windowHeight="12900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="20376" windowHeight="12096" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -118,7 +118,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -193,14 +193,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -487,16 +486,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J9"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="60.265625" customWidth="1"/>
+    <col min="1" max="1" width="60.21875" customWidth="1"/>
     <col min="2" max="2" width="38" customWidth="1"/>
     <col min="3" max="3" width="26.6640625" customWidth="1"/>
-    <col min="4" max="4" width="14.3984375" customWidth="1"/>
+    <col min="4" max="4" width="14.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -510,21 +509,21 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="3">
         <v>15.89</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
@@ -534,73 +533,67 @@
       <c r="C3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="3">
         <v>3.18</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="3">
         <v>28.99</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>14</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="3">
         <v>14.95</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>18</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="3">
         <v>8.99</v>
       </c>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.45">
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="3">
         <v>5.95</v>
       </c>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.45">
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>22</v>
       </c>
@@ -610,15 +603,12 @@
       <c r="C8" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="4">
+      <c r="D8" s="3">
         <v>3.95</v>
       </c>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="D9" s="4">
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D9" s="3">
         <f>SUM(D2:D8)</f>
         <v>81.900000000000006</v>
       </c>

</xml_diff>

<commit_message>
Fix PCB dimensions, add decoupling capacitors, and update Components list and README
</commit_message>
<xml_diff>
--- a/Components_list.xlsx
+++ b/Components_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3a2107d33766725d/Smart-Desk-Hub/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="97" documentId="11_F25DC773A252ABDACC1048B781584E2E5BDE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6FB6178F-0E14-4B57-B366-0D5AB7865750}"/>
+  <xr:revisionPtr revIDLastSave="101" documentId="11_F25DC773A252ABDACC1048B781584E2E5BDE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3F51A8E7-3099-4A46-AEB1-734ACD664854}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="20376" windowHeight="12096" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -600,7 +600,7 @@
       <c r="B8" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="4" t="s">
         <v>24</v>
       </c>
       <c r="D8" s="3">
@@ -620,8 +620,9 @@
     <hyperlink ref="C6" r:id="rId3" display="https://www.amazon.com/SATUY-INMP441-Omnidirectional-Microphone-Module/dp/B0GSZJFJVM/ref=sr_1_2_sspa?dib=eyJ2IjoiMSJ9.014Mv1cJPc5_VCF97zJYvpSDtGnmCnbujYRuowb6Dv-IzvwDJ34hmyh6RJdSO_6AKgwJIDbcnd9WzxweW7CVemb9AGH3oraR_5mIWvg59teN9d8TOoTXq1yeTzIdf7jAjRv0PDWkDYkMPultp0jMMjznzvUx2oP_L3Se7We6N5quvhwUlWfgGDNZJqy8UgnFm3Xm8-Vjjms1hRcnojbXBkeAz2RE-gpTywjitk3hL40.MTqO2y4xuc8bz4FBVKJsBeS7swbYreGqit7IFl5814I&amp;dib_tag=se&amp;keywords=inmp441%2Bi2s%2Bmicrophone&amp;qid=1791669919&amp;sr=8-2-spons&amp;sp_csd=d2lkZ2V0TmFtZT1zcF9hdGY&amp;th=1" xr:uid="{5734676C-5000-46CB-9D8B-7B73BB2DDB49}"/>
     <hyperlink ref="C5" r:id="rId4" location="technical-details" xr:uid="{A00FC8C6-F783-4EDA-99EA-AF4385B61525}"/>
     <hyperlink ref="C7" r:id="rId5" xr:uid="{87BA5DA7-E7A2-4F91-BE0E-7666654CE548}"/>
+    <hyperlink ref="C8" r:id="rId6" xr:uid="{772CB82F-B95E-4A89-9132-C8C9DD29A320}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId6"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId7"/>
 </worksheet>
 </file>
</xml_diff>